<commit_message>
ok imma keep it like this
</commit_message>
<xml_diff>
--- a/dataset/benign/codebook.xlsx
+++ b/dataset/benign/codebook.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wangcx0718\Desktop\awsflask\static\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/llukii/Desktop/School/Programming/Multimodal throat cancer/dataset/benign/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72B85D95-D40A-4581-AD83-21B98C39422D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F1DF0E7-62B4-5D4A-8296-83AC67AAD16A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="721" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" tabRatio="721" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="code book" sheetId="14" r:id="rId1"/>
@@ -131,10 +131,6 @@
     <t>用聲情形</t>
   </si>
   <si>
-    <t>VHI-10嗓音障礙指標</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>0/1/2/3</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
@@ -926,6 +922,404 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
+    <t>VHI-10嗓音障礙指標</t>
+  </si>
+  <si>
+    <r>
+      <t>1.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="新細明體"/>
+        <family val="1"/>
+        <charset val="136"/>
+      </rPr>
+      <t>聲帶息肉、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>2.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="新細明體"/>
+        <family val="1"/>
+        <charset val="136"/>
+      </rPr>
+      <t>聲帶結節、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>3.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="新細明體"/>
+        <family val="1"/>
+        <charset val="136"/>
+      </rPr>
+      <t>聲帶萎縮、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>4.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="新細明體"/>
+        <family val="1"/>
+        <charset val="136"/>
+      </rPr>
+      <t>聲帶囊腫、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>5.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="新細明體"/>
+        <family val="1"/>
+        <charset val="136"/>
+      </rPr>
+      <t>單側聲帶輕癱、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>6.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="新細明體"/>
+        <family val="1"/>
+        <charset val="136"/>
+      </rPr>
+      <t>單側聲帶麻痹、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>7.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="新細明體"/>
+        <family val="1"/>
+        <charset val="136"/>
+      </rPr>
+      <t>慢性聲帶水腫、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>8.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="新細明體"/>
+        <family val="1"/>
+        <charset val="136"/>
+      </rPr>
+      <t>聲帶溝、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>9.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="新細明體"/>
+        <family val="1"/>
+        <charset val="136"/>
+      </rPr>
+      <t>肌肉緊張性發聲異常、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>10.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="新細明體"/>
+        <family val="1"/>
+        <charset val="136"/>
+      </rPr>
+      <t>嗓音老化、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>11.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="新細明體"/>
+        <family val="1"/>
+        <charset val="136"/>
+      </rPr>
+      <t>聲帶突肉芽腫、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>12.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="新細明體"/>
+        <family val="1"/>
+        <charset val="136"/>
+      </rPr>
+      <t>纖維斑塊、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>13.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="新細明體"/>
+        <family val="1"/>
+        <charset val="136"/>
+      </rPr>
+      <t>聲帶潰瘍、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>14.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="新細明體"/>
+        <family val="1"/>
+        <charset val="136"/>
+      </rPr>
+      <t>聲帶痙攣、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>15.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="新細明體"/>
+        <family val="1"/>
+        <charset val="136"/>
+      </rPr>
+      <t>表皮異常增生、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>16.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="新細明體"/>
+        <family val="1"/>
+        <charset val="136"/>
+      </rPr>
+      <t>喉癌、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>17.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="新細明體"/>
+        <family val="1"/>
+        <charset val="136"/>
+      </rPr>
+      <t>乳突瘤、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>18.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="新細明體"/>
+        <family val="1"/>
+        <charset val="136"/>
+      </rPr>
+      <t>聲帶顫抖、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>19.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="新細明體"/>
+        <family val="1"/>
+        <charset val="136"/>
+      </rPr>
+      <t>聲帶疤痕、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>20.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="新細明體"/>
+        <family val="1"/>
+        <charset val="136"/>
+      </rPr>
+      <t>微血管增生、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>21.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="細明體"/>
+        <family val="1"/>
+        <charset val="136"/>
+      </rPr>
+      <t>正常</t>
+    </r>
+  </si>
+  <si>
     <r>
       <t>1.Polyp</t>
     </r>
@@ -1309,403 +1703,6 @@
       </rPr>
       <t>21.Normal finding</t>
     </r>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>1.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="新細明體"/>
-        <family val="1"/>
-        <charset val="136"/>
-      </rPr>
-      <t>聲帶息肉、</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>2.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="新細明體"/>
-        <family val="1"/>
-        <charset val="136"/>
-      </rPr>
-      <t>聲帶結節、</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>3.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="新細明體"/>
-        <family val="1"/>
-        <charset val="136"/>
-      </rPr>
-      <t>聲帶萎縮、</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>4.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="新細明體"/>
-        <family val="1"/>
-        <charset val="136"/>
-      </rPr>
-      <t>聲帶囊腫、</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>5.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="新細明體"/>
-        <family val="1"/>
-        <charset val="136"/>
-      </rPr>
-      <t>單側聲帶輕癱、</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>6.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="新細明體"/>
-        <family val="1"/>
-        <charset val="136"/>
-      </rPr>
-      <t>單側聲帶麻痹、</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>7.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="新細明體"/>
-        <family val="1"/>
-        <charset val="136"/>
-      </rPr>
-      <t>慢性聲帶水腫、</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>8.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="新細明體"/>
-        <family val="1"/>
-        <charset val="136"/>
-      </rPr>
-      <t>聲帶溝、</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>9.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="新細明體"/>
-        <family val="1"/>
-        <charset val="136"/>
-      </rPr>
-      <t>肌肉緊張性發聲異常、</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>10.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="新細明體"/>
-        <family val="1"/>
-        <charset val="136"/>
-      </rPr>
-      <t>嗓音老化、</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>11.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="新細明體"/>
-        <family val="1"/>
-        <charset val="136"/>
-      </rPr>
-      <t>聲帶突肉芽腫、</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>12.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="新細明體"/>
-        <family val="1"/>
-        <charset val="136"/>
-      </rPr>
-      <t>纖維斑塊、</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>13.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="新細明體"/>
-        <family val="1"/>
-        <charset val="136"/>
-      </rPr>
-      <t>聲帶潰瘍、</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>14.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="新細明體"/>
-        <family val="1"/>
-        <charset val="136"/>
-      </rPr>
-      <t>聲帶痙攣、</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>15.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="新細明體"/>
-        <family val="1"/>
-        <charset val="136"/>
-      </rPr>
-      <t>表皮異常增生、</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>16.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="新細明體"/>
-        <family val="1"/>
-        <charset val="136"/>
-      </rPr>
-      <t>喉癌、</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>17.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="新細明體"/>
-        <family val="1"/>
-        <charset val="136"/>
-      </rPr>
-      <t>乳突瘤、</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>18.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="新細明體"/>
-        <family val="1"/>
-        <charset val="136"/>
-      </rPr>
-      <t>聲帶顫抖、</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>19.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="新細明體"/>
-        <family val="1"/>
-        <charset val="136"/>
-      </rPr>
-      <t>聲帶疤痕、</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>20.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="新細明體"/>
-        <family val="1"/>
-        <charset val="136"/>
-      </rPr>
-      <t>微血管增生、</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>21.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="細明體"/>
-        <family val="1"/>
-        <charset val="136"/>
-      </rPr>
-      <t>正常</t>
-    </r>
-    <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -1713,33 +1710,33 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="176" formatCode="m&quot;月&quot;d&quot;日&quot;"/>
+    <numFmt numFmtId="164" formatCode="m&quot;月&quot;d&quot;日&quot;"/>
   </numFmts>
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="新細明體"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="新細明體"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
-      <name val="新細明體"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="136"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
-      <name val="新細明體"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <charset val="136"/>
       <scheme val="minor"/>
@@ -1891,7 +1888,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="7" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="7" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1914,7 +1911,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="一般" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="一般 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -2197,353 +2194,353 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:E28"/>
-  <sheetFormatPr defaultColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10" defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="23.5703125" style="7" customWidth="1"/>
-    <col min="2" max="2" width="29.42578125" style="8" customWidth="1"/>
-    <col min="3" max="3" width="23.28515625" style="8" customWidth="1"/>
-    <col min="4" max="4" width="42.5703125" style="8" customWidth="1"/>
-    <col min="5" max="5" width="45.28515625" style="8" customWidth="1"/>
+    <col min="1" max="1" width="23.5" style="7" customWidth="1"/>
+    <col min="2" max="2" width="29.5" style="8" customWidth="1"/>
+    <col min="3" max="3" width="23.33203125" style="8" customWidth="1"/>
+    <col min="4" max="4" width="42.5" style="8" customWidth="1"/>
+    <col min="5" max="5" width="45.33203125" style="8" customWidth="1"/>
     <col min="6" max="16384" width="10" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="18" thickBot="1">
       <c r="A1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>67</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>68</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="E1" s="2" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="138.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:5" ht="138.5" customHeight="1" thickBot="1">
       <c r="A2" s="3" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D2" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="E2" s="10" t="s">
         <v>90</v>
       </c>
-      <c r="E2" s="10" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:5" ht="18" thickBot="1">
       <c r="A3" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>4</v>
       </c>
       <c r="D3" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="E3" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="E3" s="4" t="s">
+    </row>
+    <row r="4" spans="1:5" ht="18" thickBot="1">
+      <c r="A4" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>74</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="B4" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>75</v>
       </c>
       <c r="D4" s="4"/>
       <c r="E4" s="4"/>
     </row>
-    <row r="5" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" ht="18" thickBot="1">
       <c r="A5" s="3" t="s">
         <v>5</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="18" thickBot="1">
       <c r="A6" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="18" thickBot="1">
       <c r="A7" s="3" t="s">
         <v>8</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="18" thickBot="1">
       <c r="A8" s="3" t="s">
         <v>9</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="18" thickBot="1">
       <c r="A9" s="3" t="s">
         <v>10</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="18" thickBot="1">
       <c r="A10" s="3" t="s">
         <v>11</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="18" thickBot="1">
       <c r="A11" s="3" t="s">
         <v>12</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="18" thickBot="1">
       <c r="A12" s="3" t="s">
         <v>13</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="18" thickBot="1">
       <c r="A13" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="18" thickBot="1">
       <c r="A14" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="18" thickBot="1">
       <c r="A15" s="3" t="s">
         <v>16</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="18" thickBot="1">
       <c r="A16" s="3" t="s">
         <v>17</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="18" thickBot="1">
       <c r="A17" s="3" t="s">
         <v>18</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="18" thickBot="1">
       <c r="A18" s="3" t="s">
         <v>19</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="18" thickBot="1">
       <c r="A19" s="3" t="s">
         <v>20</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="18" thickBot="1">
       <c r="A20" s="3" t="s">
         <v>21</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" ht="44.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="44.25" customHeight="1" thickBot="1">
       <c r="A21" s="3" t="s">
         <v>0</v>
       </c>
@@ -2551,126 +2548,126 @@
         <v>0</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" ht="44.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="44.25" customHeight="1" thickBot="1">
       <c r="A22" s="3" t="s">
         <v>23</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C22" s="4" t="s">
         <v>22</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" ht="44.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="44.25" customHeight="1" thickBot="1">
       <c r="A23" s="3" t="s">
         <v>24</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" ht="44.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="44.25" customHeight="1" thickBot="1">
       <c r="A24" s="3" t="s">
         <v>25</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C24" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="E24" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="D24" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="E24" s="4" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" ht="44.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="25" spans="1:5" ht="44.25" customHeight="1" thickBot="1">
       <c r="A25" s="3" t="s">
         <v>26</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" ht="44.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="44.25" customHeight="1" thickBot="1">
       <c r="A26" s="3" t="s">
         <v>27</v>
       </c>
       <c r="B26" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D26" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="C26" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="D26" s="4" t="s">
-        <v>85</v>
-      </c>
       <c r="E26" s="4" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" ht="44.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="44.25" customHeight="1" thickBot="1">
       <c r="A27" s="3" t="s">
         <v>28</v>
       </c>
       <c r="B27" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="44.25" customHeight="1" thickBot="1">
+      <c r="A28" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="B28" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="C27" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="D27" s="4" t="s">
+      <c r="C28" s="4" t="s">
         <v>86</v>
-      </c>
-      <c r="E27" s="4" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" ht="44.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="B28" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="C28" s="4" t="s">
-        <v>87</v>
       </c>
       <c r="D28" s="4"/>
       <c r="E28" s="4"/>

</xml_diff>